<commit_message>
question 3 state diagram
</commit_message>
<xml_diff>
--- a/AI Audit Log_LeTrongPhuc.xlsx
+++ b/AI Audit Log_LeTrongPhuc.xlsx
@@ -1,95 +1,91 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Education\Summer2026\Github\ai-audit-log-trongphuc207\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06BBB08A-1653-4BFE-B60C-D48E2A0E1583}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="5"/>
   </bookViews>
   <sheets>
-    <sheet name="Week 1" sheetId="1" r:id="rId1"/>
-    <sheet name="Week 2" sheetId="2" r:id="rId2"/>
-    <sheet name="Week 3" sheetId="3" r:id="rId3"/>
-    <sheet name="Week 4" sheetId="4" r:id="rId4"/>
-    <sheet name="Week 5" sheetId="5" r:id="rId5"/>
-    <sheet name="Week 6" sheetId="6" r:id="rId6"/>
-    <sheet name="Week 7 " sheetId="7" r:id="rId7"/>
-    <sheet name="Week 8" sheetId="8" r:id="rId8"/>
-    <sheet name="Week 9" sheetId="9" r:id="rId9"/>
-    <sheet name="Week 10" sheetId="10" r:id="rId10"/>
+    <sheet name="Week 1" sheetId="1" state="visible" r:id="rId2"/>
+    <sheet name="Week 2" sheetId="2" state="visible" r:id="rId3"/>
+    <sheet name="Week 3" sheetId="3" state="visible" r:id="rId4"/>
+    <sheet name="Week 4" sheetId="4" state="visible" r:id="rId5"/>
+    <sheet name="Week 5" sheetId="5" state="visible" r:id="rId6"/>
+    <sheet name="Week 6" sheetId="6" state="visible" r:id="rId7"/>
+    <sheet name="Week 7 " sheetId="7" state="visible" r:id="rId8"/>
+    <sheet name="Week 8" sheetId="8" state="visible" r:id="rId9"/>
+    <sheet name="Week 9" sheetId="9" state="visible" r:id="rId10"/>
+    <sheet name="Week 10" sheetId="10" state="visible" r:id="rId11"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr/>
+  <extLst>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{D0CA8CA8-9F24-4464-BF8E-62219DCF47F9}"/>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="34">
   <si>
     <t>STT</t>
   </si>
   <si>
-    <t>Giai đoạn/Thành phần DTC</t>
-  </si>
-  <si>
-    <t>Nội dung Prompt (Câu lệnh)</t>
-  </si>
-  <si>
-    <t>Phản hồi của AI &amp; Quyết định của người học (Reflection)</t>
-  </si>
-  <si>
-    <t>Ví dụ: Abstraction</t>
-  </si>
-  <si>
-    <t>“Tôi cần quản lý thông tin sinh viên cho app quản lý điểm. Hãy liệt kê các thuộc tính cần thiết."</t>
-  </si>
-  <si>
-    <t>Phản hồi: AI liệt kê 20 thuộc tính.
+    <t xml:space="preserve">Giai đoạn/Thành phần DTC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nội dung Prompt (Câu lệnh)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Phản hồi của AI &amp; Quyết định của người học (Reflection)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ví dụ: Abstraction</t>
+  </si>
+  <si>
+    <t xml:space="preserve">“Tôi cần quản lý thông tin sinh viên cho app quản lý điểm. Hãy liệt kê các thuộc tính cần thiết."</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Phản hồi: AI liệt kê 20 thuộc tính.
  Quyết định: Tôi chỉ chọn 10 thuộc tính liên quan đến chức năng đang được yêu cầu từ ứng dụng (CCCD, địa chỉ...) và lược bỏ 10 thuộc tính học thuật vì phù hợp với yêu cầu của ứng dụng</t>
   </si>
   <si>
-    <t>Ví dụ: Process/Algorithm</t>
-  </si>
-  <si>
-    <t>"Viết hàm C sắp xếp mảng sinh viên theo điểm số bằng Selection Sort."</t>
-  </si>
-  <si>
-    <t>Phản hồi: AI cung cấp code mẫu.
+    <t xml:space="preserve">Ví dụ: Process/Algorithm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"Viết hàm C sắp xếp mảng sinh viên theo điểm số bằng Selection Sort."</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Phản hồi: AI cung cấp code mẫu.
  Kiểm chứng: Tôi nhận thấy code AI chưa xử lý trường hợp mảng rỗng (Oversimplification). Tôi đã yêu cầu AI tối ưu lại và tự tay bổ sung điều kiện kiểm tra lỗi.</t>
   </si>
   <si>
-    <t>Ví dụ: Pattern Recognition</t>
-  </si>
-  <si>
-    <t>“So sánh các giải thuật CPU scheduling: FCFS, SJF, Round Robin, Priority. Giải thuật nào tốt nhất?”</t>
-  </si>
-  <si>
-    <t>Phản hồi: AI response Round Robin là “tốt nhất” vì cân bằng giữa throughput và fairness.
+    <t xml:space="preserve">Ví dụ: Pattern Recognition</t>
+  </si>
+  <si>
+    <t xml:space="preserve">“So sánh các giải thuật CPU scheduling: FCFS, SJF, Round Robin, Priority. Giải thuật nào tốt nhất?”</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Phản hồi: AI response Round Robin là “tốt nhất” vì cân bằng giữa throughput và fairness.
  Kiểm chứng: AI đưa kết luận sai – không có giải thuật “tốt nhất” tuyệt đối (Hallucination). Mỗi giải thuật phù hợp với tình huống/context khác nhau.</t>
   </si>
   <si>
-    <t>Ví dụ: Pattern Recognition + Literature Review</t>
-  </si>
-  <si>
-    <t>“Tóm tắt 5 bài báo gần đây nhất về anomaly detection trong IoT sensor data.”</t>
-  </si>
-  <si>
-    <t>Phản hồi: AI tóm tắt 5 papers với tên tác giả, năm xuất bản và tóm tắt nội dung.
+    <t xml:space="preserve">Ví dụ: Pattern Recognition + Literature Review</t>
+  </si>
+  <si>
+    <t xml:space="preserve">“Tóm tắt 5 bài báo gần đây nhất về anomaly detection trong IoT sensor data.”</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Phản hồi: AI tóm tắt 5 papers với tên tác giả, năm xuất bản và tóm tắt nội dung.
  Kiểm chứng: Tìm trên Google Scholar: 2/5 papers AI nêu là không tồn tại (fabrication). Tôi đã thay bằng 2 papers mà tôi đã tìm kiếm trên research gates và đã kiểm chứng trên google scholar.</t>
   </si>
   <si>
-    <t>Phân tích Use Case</t>
-  </si>
-  <si>
-    <t>Use case là gì và các thành phần trong use case</t>
-  </si>
-  <si>
-    <t>Biểu diễn sơ đồ chức năng của hệ thống. Mỗi use case mô tả chức năng mà hệ thống cần phải có xét từ góc độ người dùng.
+    <t xml:space="preserve">Phân tích Use Case</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Use case là gì và các thành phần trong use case</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Biểu diễn sơ đồ chức năng của hệ thống. Mỗi use case mô tả chức năng mà hệ thống cần phải có xét từ góc độ người dùng.
 Actor: Là người dùng hoặc đối tượng bên ngoài có khả năng tương tác với hệ thống.
 Use Case: Là các chức năng mà actor sử dụng để tương tác với hệ thống.
 Communication Link: Là đường kết nối giữa Actor và Use Case, thể hiện sự tương tác.
@@ -104,74 +100,83 @@
 Bước 3: Xác định mối quan hệ</t>
   </si>
   <si>
-    <t>Tìm kiếm chức năng của Manager</t>
-  </si>
-  <si>
-    <t>Manager có những chức năng gì, hãy liệt kê giúp tôi</t>
-  </si>
-  <si>
-    <t>Phản hồi: AI đề xuất các chức năng gồm Log In, Manage Menu, Add Menu Item, Update Menu Item, Remove Menu Item, Manage Employees, View Revenue Reports và Manage Promotions. Ngoài ra AI còn gợi ý sử dụng quan hệ include giữa Manage Menu với Add/Update/Remove Menu Item.</t>
-  </si>
-  <si>
-    <t>Tìm kiếm chức năng của Barista</t>
-  </si>
-  <si>
-    <t>Tìm kiếm chức năng của Waiter</t>
-  </si>
-  <si>
-    <t>Tìm kiếm chức năng của Cashier</t>
-  </si>
-  <si>
-    <t>Cashier có những chức năng gì, hãy liệt kê giúp tôi</t>
-  </si>
-  <si>
-    <t>Waiter có những chức năng gì, hãy liệt kê giúp tôi</t>
-  </si>
-  <si>
-    <t>Barista có những chức năng gì, hãy liệt kê giúp tôi</t>
-  </si>
-  <si>
-    <t>Phản hồi: AI liệt kê các chức năng gồm View Pending Orders, Start Preparing Order, Update Order Status, Mark Order as Ready, Report Out-of-Stock Ingredients và View Daily Orders. Ngoài ra AI còn đề xuất include relationship giữa Start Preparing Order và View Pending Orders.</t>
-  </si>
-  <si>
-    <t>Phản hồi: AI đề xuất các chức năng gồm View Menu, Create Order, Modify Order, Cancel Order, Assign Table, Send Order to Barista và Update Table Status. AI cũng đề xuất include relationship giữa Create Order và View Menu, cùng extend relationship với Modify Order, Cancel Order và Assign Table.</t>
-  </si>
-  <si>
-    <t>Phản hồi: AI đề xuất các chức năng gồm Process Payment, Generate Invoice, Print Receipt, Apply Discount, Verify Membership, Redeem Reward Points, Refund Payment và View Payment History. Ngoài ra AI còn gợi ý include relationship giữa Process Payment với Generate Invoice và Verify Membership; extend relationship với Apply Discount và Refund Payment.</t>
+    <t xml:space="preserve">Tìm kiếm chức năng của Manager</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Manager có những chức năng gì, hãy liệt kê giúp tôi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Phản hồi: AI đề xuất các chức năng gồm Log In, Manage Menu, Add Menu Item, Update Menu Item, Remove Menu Item, Manage Employees, View Revenue Reports và Manage Promotions. Ngoài ra AI còn gợi ý sử dụng quan hệ include giữa Manage Menu với Add/Update/Remove Menu Item.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tìm kiếm chức năng của Barista</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Barista có những chức năng gì, hãy liệt kê giúp tôi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Phản hồi: AI liệt kê các chức năng gồm View Pending Orders, Start Preparing Order, Update Order Status, Mark Order as Ready, Report Out-of-Stock Ingredients và View Daily Orders. Ngoài ra AI còn đề xuất include relationship giữa Start Preparing Order và View Pending Orders.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tìm kiếm chức năng của Waiter</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Waiter có những chức năng gì, hãy liệt kê giúp tôi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Phản hồi: AI đề xuất các chức năng gồm View Menu, Create Order, Modify Order, Cancel Order, Assign Table, Send Order to Barista và Update Table Status. AI cũng đề xuất include relationship giữa Create Order và View Menu, cùng extend relationship với Modify Order, Cancel Order và Assign Table.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tìm kiếm chức năng của Cashier</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cashier có những chức năng gì, hãy liệt kê giúp tôi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Phản hồi: AI đề xuất các chức năng gồm Process Payment, Generate Invoice, Print Receipt, Apply Discount, Verify Membership, Redeem Reward Points, Refund Payment và View Payment History. Ngoài ra AI còn gợi ý include relationship giữa Process Payment với Generate Invoice và Verify Membership; extend relationship với Apply Discount và Refund Payment.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thiết kế State Diagram</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hãy thiết kế UML State Diagram cho thực thể Order trong hệ thống quản lý nhà hàng Vincom Food Court. Order phải trải qua các trạng thái: Created, Confirmed, Paid, Preparing, ReadyToServe, Served và Completed. Bổ sung các trường hợp ngoại lệ như PaymentFailed và Cancelled. Hiển thị đầy đủ trạng thái bắt đầu (Initial State), trạng thái kết thúc (Final State) và các sự kiện kích hoạt chuyển trạng thái như confirmOrder, paySuccess, payFail, startCooking, finishCooking, serveOrder và closeOrder.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AI đề xuất State Diagram mô tả đầy đủ vòng đời của Order từ khi khách hàng tạo đơn đến khi hoàn tất phục vụ. AI bổ sung hai nhánh ngoại lệ là PaymentFailed và Cancelled để xử lý các trường hợp thanh toán thất bại hoặc hủy đơn. Sau khi xem xét kết quả, người học quyết định giữ lại toàn bộ các trạng thái chính vì phù hợp với yêu cầu đề bài. Đồng thời, người học chỉnh sửa bố cục sơ đồ để các luồng thành công và thất bại được tách biệt, dễ theo dõi hơn. Người học cũng lựa chọn chỉ sử dụng một trạng thái Cancelled duy nhất thay vì lặp lại nhiều lần nhằm tuân thủ nguyên tắc UML và làm cho sơ đồ rõ ràng, dễ đọc hơn. Cuối cùng, sơ đồ được hoàn thiện và sử dụng làm kết quả chính thức cho bài thực hành.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="5">
     <font>
-      <sz val="10"/>
-      <color rgb="FF000000"/>
+      <sz val="10.000000"/>
+      <color indexed="64"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
+      <sz val="11.000000"/>
+      <color indexed="64"/>
       <name val="&quot;Aptos Narrow&quot;"/>
     </font>
     <font>
       <b/>
-      <sz val="10"/>
+      <sz val="10.000000"/>
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
+      <sz val="11.000000"/>
+      <color indexed="64"/>
       <name val="&quot;Aptos Narrow&quot;"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
+      <sz val="11.000000"/>
+      <color indexed="64"/>
       <name val="Arial"/>
     </font>
   </fonts>
@@ -184,75 +189,84 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFFF"/>
-        <bgColor rgb="FFFFFFFF"/>
+        <fgColor indexed="65"/>
+        <bgColor indexed="65"/>
       </patternFill>
     </fill>
   </fills>
   <borders count="2">
     <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
     </border>
     <border>
       <left style="thin">
-        <color rgb="FF000000"/>
+        <color indexed="64"/>
       </left>
       <right style="thin">
-        <color rgb="FF000000"/>
+        <color indexed="64"/>
       </right>
       <top style="thin">
-        <color rgb="FF000000"/>
+        <color indexed="64"/>
       </top>
       <bottom style="thin">
-        <color rgb="FF000000"/>
+        <color indexed="64"/>
       </bottom>
-      <diagonal/>
+      <diagonal style="none"/>
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="13">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+  <cellXfs count="16">
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
+    <xf fontId="1" fillId="2" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf fontId="2" fillId="2" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="3" fillId="2" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="3" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="4" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="4" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="3" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="3" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="1" fillId="2" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="3" fillId="2" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="4" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="4" fillId="2" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf fontId="1" fillId="2" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf fontId="3" fillId="2" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf fontId="4" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -271,8 +285,327 @@
 </styleSheet>
 </file>
 
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math" xmlns:w="http://schemas.openxmlformats.org/wordprocessingml/2006/main">
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="7400917" cy="5151119"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="1692984230" name=""/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill rotWithShape="1">
+        <a:blip r:embed="rId1"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="7400917" cy="5151119"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/theme/theme.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+  <a:themeElements>
+    <a:clrScheme name="Office">
+      <a:dk1>
+        <a:sysClr val="windowText" lastClr="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="1F497D"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="EEECE1"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="4F81BD"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="C0504D"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="9BBB59"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="8064A2"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="4BACC6"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="F79646"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="0000FF"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="800080"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Cambria"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ ゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Angsana New"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Calibri"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ 明朝"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Cordia New"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme name="Office">
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="50000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="35000">
+              <a:schemeClr val="phClr">
+                <a:tint val="37000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:tint val="15000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="1"/>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:shade val="51000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="80000">
+              <a:schemeClr val="phClr">
+                <a:shade val="93000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="94000"/>
+                <a:satMod val="135000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="0"/>
+        </a:gradFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr">
+              <a:shade val="95000"/>
+              <a:satMod val="105000"/>
+            </a:schemeClr>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="38000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+          <a:scene3d>
+            <a:camera prst="orthographicFront">
+              <a:rot lat="0" lon="0" rev="0"/>
+            </a:camera>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
+            </a:lightRig>
+          </a:scene3d>
+          <a:sp3d>
+            <a:bevelT w="63500" h="25400"/>
+          </a:sp3d>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="40000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="40000">
+              <a:schemeClr val="phClr">
+                <a:tint val="45000"/>
+                <a:shade val="99000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="20000"/>
+                <a:satMod val="255000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
+          </a:path>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="80000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="30000"/>
+                <a:satMod val="200000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
+          </a:path>
+        </a:gradFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
+</a:theme>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:p="http://schemas.openxmlformats.org/presentationml/2006/main" name="Sheets">
   <a:themeElements>
     <a:clrScheme name="Sheets">
       <a:dk1>
@@ -329,7 +662,7 @@
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill>
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -355,7 +688,7 @@
           </a:gsLst>
           <a:lin ang="5400000" scaled="0"/>
         </a:gradFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill>
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -432,7 +765,7 @@
             <a:satMod val="170000"/>
           </a:schemeClr>
         </a:solidFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill>
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -463,25 +796,24 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetPr>
-    <outlinePr summaryBelow="0" summaryRight="0"/>
+    <outlinePr applyStyles="0" summaryBelow="0" summaryRight="0" showOutlineSymbols="1"/>
+    <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
   <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
-    <col min="2" max="2" width="28.6640625" customWidth="1"/>
-    <col min="3" max="3" width="33.88671875" customWidth="1"/>
-    <col min="4" max="4" width="82.109375" customWidth="1"/>
-    <col min="5" max="5" width="33.6640625" customWidth="1"/>
+    <col customWidth="1" min="2" max="2" width="28.6640625"/>
+    <col customWidth="1" min="3" max="3" width="33.88671875"/>
+    <col customWidth="1" min="4" max="4" width="82.109375"/>
+    <col customWidth="1" min="5" max="5" width="33.6640625"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="16.2" customHeight="1">
+    <row r="1" ht="16.199999999999999" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -496,7 +828,7 @@
       </c>
       <c r="E1" s="2"/>
     </row>
-    <row r="2" spans="1:5" ht="57.6" customHeight="1">
+    <row r="2" ht="57.600000000000001" customHeight="1">
       <c r="A2" s="3">
         <v>1</v>
       </c>
@@ -510,7 +842,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="53.4" customHeight="1">
+    <row r="3" ht="53.399999999999999" customHeight="1">
       <c r="A3" s="3">
         <v>2</v>
       </c>
@@ -524,7 +856,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="57" customHeight="1">
+    <row r="4" ht="57" customHeight="1">
       <c r="A4" s="3">
         <v>3</v>
       </c>
@@ -538,7 +870,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="64.2" customHeight="1">
+    <row r="5" ht="64.200000000000003" customHeight="1">
       <c r="A5" s="3">
         <v>4</v>
       </c>
@@ -553,37 +885,43 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetPr>
-    <outlinePr summaryBelow="0" summaryRight="0"/>
+    <outlinePr applyStyles="0" summaryBelow="0" summaryRight="0" showOutlineSymbols="1"/>
+    <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1"/>
   <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
   <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetPr>
-    <outlinePr summaryBelow="0" summaryRight="0"/>
+    <outlinePr applyStyles="0" summaryBelow="0" summaryRight="0" showOutlineSymbols="1"/>
+    <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
   <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
-    <col min="2" max="2" width="34.21875" customWidth="1"/>
-    <col min="3" max="3" width="35.44140625" customWidth="1"/>
-    <col min="4" max="4" width="77.21875" customWidth="1"/>
-    <col min="5" max="5" width="29" customWidth="1"/>
+    <col customWidth="1" min="2" max="2" width="34.21875"/>
+    <col customWidth="1" min="3" max="3" width="35.44140625"/>
+    <col customWidth="1" min="4" max="4" width="77.21875"/>
+    <col customWidth="1" min="5" max="5" width="29"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="13.8">
+    <row r="1" ht="13.800000000000001">
       <c r="A1" s="9" t="s">
         <v>0</v>
       </c>
@@ -598,7 +936,7 @@
       </c>
       <c r="E1" s="2"/>
     </row>
-    <row r="2" spans="1:5" ht="250.2" customHeight="1">
+    <row r="2" ht="250.19999999999999" customHeight="1">
       <c r="A2" s="10">
         <v>1</v>
       </c>
@@ -612,7 +950,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="67.2" customHeight="1">
+    <row r="3" ht="67.200000000000003" customHeight="1">
       <c r="A3" s="10">
         <v>3</v>
       </c>
@@ -626,7 +964,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="96" customHeight="1">
+    <row r="4" ht="96" customHeight="1">
       <c r="A4" s="12">
         <v>4</v>
       </c>
@@ -634,125 +972,184 @@
         <v>22</v>
       </c>
       <c r="C4" s="11" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="D4" s="11" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" ht="90.6" customHeight="1">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="5" ht="90.599999999999994" customHeight="1">
       <c r="A5" s="10">
         <v>5</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C5" s="11" t="s">
         <v>26</v>
       </c>
       <c r="D5" s="11" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" ht="73.2" customHeight="1">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="6" ht="73.200000000000003" customHeight="1">
       <c r="A6" s="12">
         <v>6</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="D6" s="11" t="s">
         <v>30</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetPr>
-    <outlinePr summaryBelow="0" summaryRight="0"/>
+    <outlinePr applyStyles="0" summaryBelow="0" summaryRight="0" showOutlineSymbols="1"/>
+    <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1"/>
   <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
   <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetPr>
-    <outlinePr summaryBelow="0" summaryRight="0"/>
+    <outlinePr applyStyles="0" summaryBelow="0" summaryRight="0" showOutlineSymbols="1"/>
+    <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1"/>
   <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
   <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetPr>
-    <outlinePr summaryBelow="0" summaryRight="0"/>
+    <outlinePr applyStyles="0" summaryBelow="0" summaryRight="0" showOutlineSymbols="1"/>
+    <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1"/>
   <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
   <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetPr>
-    <outlinePr summaryBelow="0" summaryRight="0"/>
+    <outlinePr applyStyles="0" summaryBelow="0" summaryRight="0" showOutlineSymbols="1"/>
+    <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1"/>
+  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
+  <cols>
+    <col customWidth="1" min="2" max="2" width="35.421875"/>
+    <col customWidth="1" min="3" max="3" width="64.00390625"/>
+    <col customWidth="1" min="4" max="4" width="80.00390625"/>
+  </cols>
+  <sheetData>
+    <row r="28" ht="60" customHeight="1">
+      <c r="A28" s="13" t="s">
+        <v>0</v>
+      </c>
+      <c r="B28" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="C28" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="D28" s="13" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="29" ht="215.40000000000001" customHeight="1">
+      <c r="A29" s="14">
+        <v>1</v>
+      </c>
+      <c r="B29" s="15" t="s">
+        <v>31</v>
+      </c>
+      <c r="C29" s="11" t="s">
+        <v>32</v>
+      </c>
+      <c r="D29" s="11" t="s">
+        <v>33</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
+  <sheetPr>
+    <outlinePr applyStyles="0" summaryBelow="0" summaryRight="0" showOutlineSymbols="1"/>
+    <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
+  </sheetPr>
   <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
   <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetPr>
-    <outlinePr summaryBelow="0" summaryRight="0"/>
+    <outlinePr applyStyles="0" summaryBelow="0" summaryRight="0" showOutlineSymbols="1"/>
+    <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1"/>
   <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
   <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetPr>
-    <outlinePr summaryBelow="0" summaryRight="0"/>
+    <outlinePr applyStyles="0" summaryBelow="0" summaryRight="0" showOutlineSymbols="1"/>
+    <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1"/>
   <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
   <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
-  <sheetPr>
-    <outlinePr summaryBelow="0" summaryRight="0"/>
-  </sheetPr>
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
 </worksheet>
 </file>
</xml_diff>